<commit_message>
update data for "Blocco 2"
</commit_message>
<xml_diff>
--- a/public/fisiorock_block2.xlsx
+++ b/public/fisiorock_block2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\U82739\Documents\Personale\FisioRock\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\U82739\workspace\fisiorock-workouts\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4B09C4-63ED-4AE8-92A9-EFBCEF82BCFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF060C01-6097-4731-A5DD-717B1548A123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="6960" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{3CC28C5F-FDBF-9A46-9F27-14F8E8FE9680}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="3" xr2:uid="{3CC28C5F-FDBF-9A46-9F27-14F8E8FE9680}"/>
   </bookViews>
   <sheets>
     <sheet name="Warm Up" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="78">
   <si>
     <t>N°</t>
   </si>
@@ -318,6 +318,9 @@
   </si>
   <si>
     <t>10</t>
+  </si>
+  <si>
+    <t>3-5</t>
   </si>
 </sst>
 </file>
@@ -678,6 +681,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -701,15 +713,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1061,15 +1064,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
     </row>
     <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
@@ -1331,17 +1334,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
@@ -1480,17 +1483,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
@@ -1532,7 +1535,7 @@
         <v>3</v>
       </c>
       <c r="D3" s="21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" s="19">
         <v>1</v>
@@ -1561,7 +1564,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E4" s="19">
         <v>1</v>
@@ -1590,7 +1593,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" s="19">
         <v>1</v>
@@ -1638,13 +1641,13 @@
       <c r="B7" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="24">
-        <v>3</v>
-      </c>
-      <c r="D7" s="53" t="s">
+      <c r="C7" s="45" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="E7" s="54">
+      <c r="E7" s="46">
         <v>3</v>
       </c>
       <c r="F7" s="26"/>
@@ -1793,17 +1796,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
@@ -1845,7 +1848,7 @@
         <v>3</v>
       </c>
       <c r="D3" s="21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" s="19">
         <v>1</v>
@@ -1874,7 +1877,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E4" s="19">
         <v>1</v>
@@ -1903,7 +1906,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" s="19">
         <v>1</v>
@@ -1954,7 +1957,7 @@
       <c r="C7" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="D7" s="55">
+      <c r="D7" s="47">
         <v>3</v>
       </c>
       <c r="E7" s="26"/>
@@ -2111,17 +2114,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
@@ -2283,17 +2286,17 @@
       <c r="I8" s="40"/>
     </row>
     <row r="9" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="50" t="s">
+      <c r="A9" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="B9" s="51"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
-      <c r="I9" s="52"/>
+      <c r="B9" s="54"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="54"/>
+      <c r="G9" s="54"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="55"/>
     </row>
     <row r="10" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="41">
@@ -2426,17 +2429,17 @@
       <c r="I15" s="40"/>
     </row>
     <row r="16" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="50" t="s">
+      <c r="A16" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="51"/>
-      <c r="C16" s="51"/>
-      <c r="D16" s="51"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="51"/>
-      <c r="G16" s="51"/>
-      <c r="H16" s="51"/>
-      <c r="I16" s="52"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="54"/>
+      <c r="G16" s="54"/>
+      <c r="H16" s="54"/>
+      <c r="I16" s="55"/>
     </row>
     <row r="17" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="41">

</xml_diff>